<commit_message>
Forecast/target comparisons and a decluttered professional summary
Files without prior-year months now compare full-year outlook
(actuals + forecast) against the FY target column: variance, variance
% and RAG across hero tiles, KPI cards, the left-pane KPI list,
breakdown tables and Excel exports all switch to that basis, with
labels following. FY outlook, FY target and variance-vs-target join
the measure dropdowns in the Mix analysis and chart builder for such
files. The KPI summary is decluttered: compact single-line cards
capped at the top six by materiality with a show-all toggle, tighter
grid, hover-hint instead of a hint paragraph, and basis-aware page
copy. The CIB sample generator now scales quarters, YTD and FY
columns realistically.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/sample/IWPB_SG_Driller_CIB_style.xlsx
+++ b/iwpb-sg-dashboard/sample/IWPB_SG_Driller_CIB_style.xlsx
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>12.4</v>
+        <v>37.3</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -886,13 +886,13 @@
         <v>0</v>
       </c>
       <c r="AG6" t="n">
-        <v>6.5</v>
+        <v>77.8</v>
       </c>
       <c r="AH6" t="n">
-        <v>29.2</v>
+        <v>350.9</v>
       </c>
       <c r="AI6" t="n">
-        <v>9.4</v>
+        <v>112.5</v>
       </c>
     </row>
     <row r="7">
@@ -1011,16 +1011,16 @@
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>11.3</v>
+        <v>33.8</v>
       </c>
       <c r="AD7" t="n">
-        <v>11.6</v>
+        <v>34.8</v>
       </c>
       <c r="AE7" t="n">
-        <v>13.9</v>
+        <v>41.6</v>
       </c>
       <c r="AF7" t="n">
-        <v>12</v>
+        <v>71.8</v>
       </c>
       <c r="AG7" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>6.7</v>
+        <v>20</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -1160,13 +1160,13 @@
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>10.3</v>
+        <v>123.2</v>
       </c>
       <c r="AH8" t="n">
         <v>0</v>
       </c>
       <c r="AI8" t="n">
-        <v>5.5</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="9">
@@ -1282,7 +1282,7 @@
         <v>19.2</v>
       </c>
       <c r="AB9" t="n">
-        <v>34.7</v>
+        <v>104</v>
       </c>
       <c r="AC9" t="n">
         <v>0</v>
@@ -1291,16 +1291,16 @@
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>25.1</v>
+        <v>75.2</v>
       </c>
       <c r="AF9" t="n">
-        <v>22.3</v>
+        <v>133.6</v>
       </c>
       <c r="AG9" t="n">
-        <v>15</v>
+        <v>180.2</v>
       </c>
       <c r="AH9" t="n">
-        <v>15.6</v>
+        <v>187.5</v>
       </c>
       <c r="AI9" t="n">
         <v>0</v>
@@ -1419,28 +1419,28 @@
         <v>17.6</v>
       </c>
       <c r="AB10" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>17.1</v>
+        <v>51.3</v>
       </c>
       <c r="AE10" t="n">
-        <v>2.6</v>
+        <v>7.9</v>
       </c>
       <c r="AF10" t="n">
-        <v>22.8</v>
+        <v>136.6</v>
       </c>
       <c r="AG10" t="n">
-        <v>2.7</v>
+        <v>31.9</v>
       </c>
       <c r="AH10" t="n">
-        <v>30.5</v>
+        <v>365.6</v>
       </c>
       <c r="AI10" t="n">
-        <v>9.699999999999999</v>
+        <v>116.4</v>
       </c>
     </row>
     <row r="11">
@@ -1556,7 +1556,7 @@
         <v>35.9</v>
       </c>
       <c r="AB11" t="n">
-        <v>11.2</v>
+        <v>33.6</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -1565,19 +1565,19 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>14.1</v>
+        <v>42.3</v>
       </c>
       <c r="AF11" t="n">
-        <v>37.2</v>
+        <v>222.9</v>
       </c>
       <c r="AG11" t="n">
-        <v>42.8</v>
+        <v>513.1</v>
       </c>
       <c r="AH11" t="n">
-        <v>7.4</v>
+        <v>88.2</v>
       </c>
       <c r="AI11" t="n">
-        <v>45.1</v>
+        <v>541.3</v>
       </c>
     </row>
     <row r="12">
@@ -1693,25 +1693,25 @@
         <v>5.7</v>
       </c>
       <c r="AB12" t="n">
-        <v>8.9</v>
+        <v>26.6</v>
       </c>
       <c r="AC12" t="n">
-        <v>7.4</v>
+        <v>22.3</v>
       </c>
       <c r="AD12" t="n">
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>9.1</v>
+        <v>27.4</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>6</v>
+        <v>72.3</v>
       </c>
       <c r="AH12" t="n">
-        <v>7.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="AI12" t="n">
         <v>0</v>
@@ -1830,28 +1830,28 @@
         <v>1.5</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.8</v>
+        <v>5.5</v>
       </c>
       <c r="AD13" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.3</v>
+        <v>1.9</v>
       </c>
       <c r="AG13" t="n">
-        <v>2.6</v>
+        <v>30.7</v>
       </c>
       <c r="AH13" t="n">
-        <v>2.6</v>
+        <v>31.1</v>
       </c>
       <c r="AI13" t="n">
-        <v>1.2</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="14">
@@ -1967,28 +1967,28 @@
         <v>11.2</v>
       </c>
       <c r="AB14" t="n">
-        <v>25.3</v>
+        <v>75.8</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>53.2</v>
+        <v>159.7</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>41.1</v>
+        <v>246.5</v>
       </c>
       <c r="AG14" t="n">
-        <v>36.7</v>
+        <v>440.4</v>
       </c>
       <c r="AH14" t="n">
-        <v>37.7</v>
+        <v>452.4</v>
       </c>
       <c r="AI14" t="n">
-        <v>42.6</v>
+        <v>511</v>
       </c>
     </row>
     <row r="15">
@@ -2104,28 +2104,28 @@
         <v>0</v>
       </c>
       <c r="AB15" t="n">
-        <v>18.6</v>
+        <v>55.8</v>
       </c>
       <c r="AC15" t="n">
-        <v>18.7</v>
+        <v>56.1</v>
       </c>
       <c r="AD15" t="n">
-        <v>19</v>
+        <v>57.1</v>
       </c>
       <c r="AE15" t="n">
-        <v>8.4</v>
+        <v>25.3</v>
       </c>
       <c r="AF15" t="n">
-        <v>28.7</v>
+        <v>172.2</v>
       </c>
       <c r="AG15" t="n">
-        <v>19.1</v>
+        <v>229.5</v>
       </c>
       <c r="AH15" t="n">
-        <v>17.4</v>
+        <v>209.1</v>
       </c>
       <c r="AI15" t="n">
-        <v>37.9</v>
+        <v>454.4</v>
       </c>
     </row>
     <row r="16">
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="AC16" t="n">
-        <v>26.1</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AD16" t="n">
         <v>0</v>
@@ -2253,13 +2253,13 @@
         <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>25.9</v>
+        <v>155.6</v>
       </c>
       <c r="AG16" t="n">
-        <v>13.7</v>
+        <v>164.9</v>
       </c>
       <c r="AH16" t="n">
-        <v>25.1</v>
+        <v>301.3</v>
       </c>
       <c r="AI16" t="n">
         <v>0</v>
@@ -2378,28 +2378,28 @@
         <v>0</v>
       </c>
       <c r="AB17" t="n">
-        <v>9.699999999999999</v>
+        <v>29</v>
       </c>
       <c r="AC17" t="n">
         <v>0</v>
       </c>
       <c r="AD17" t="n">
-        <v>34.2</v>
+        <v>102.5</v>
       </c>
       <c r="AE17" t="n">
-        <v>32.4</v>
+        <v>97.3</v>
       </c>
       <c r="AF17" t="n">
-        <v>26.4</v>
+        <v>158.3</v>
       </c>
       <c r="AG17" t="n">
-        <v>30.6</v>
+        <v>367.2</v>
       </c>
       <c r="AH17" t="n">
-        <v>24.6</v>
+        <v>295.4</v>
       </c>
       <c r="AI17" t="n">
-        <v>10</v>
+        <v>120.4</v>
       </c>
     </row>
     <row r="18">
@@ -2515,28 +2515,28 @@
         <v>0</v>
       </c>
       <c r="AB18" t="n">
-        <v>25.9</v>
+        <v>77.8</v>
       </c>
       <c r="AC18" t="n">
-        <v>25</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AD18" t="n">
-        <v>29.5</v>
+        <v>88.5</v>
       </c>
       <c r="AE18" t="n">
-        <v>22.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AF18" t="n">
-        <v>25.8</v>
+        <v>155.1</v>
       </c>
       <c r="AG18" t="n">
         <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>25.3</v>
+        <v>303.4</v>
       </c>
       <c r="AI18" t="n">
-        <v>8.6</v>
+        <v>103.2</v>
       </c>
     </row>
     <row r="19">
@@ -2652,25 +2652,25 @@
         <v>17</v>
       </c>
       <c r="AB19" t="n">
-        <v>13.3</v>
+        <v>39.9</v>
       </c>
       <c r="AC19" t="n">
-        <v>13.3</v>
+        <v>40</v>
       </c>
       <c r="AD19" t="n">
-        <v>11.6</v>
+        <v>34.8</v>
       </c>
       <c r="AE19" t="n">
-        <v>25.2</v>
+        <v>75.5</v>
       </c>
       <c r="AF19" t="n">
-        <v>5.2</v>
+        <v>31.3</v>
       </c>
       <c r="AG19" t="n">
-        <v>35.1</v>
+        <v>420.8</v>
       </c>
       <c r="AH19" t="n">
-        <v>18.2</v>
+        <v>217.9</v>
       </c>
       <c r="AI19" t="n">
         <v>0</v>
@@ -2795,14 +2795,14 @@
         <v>-27.1</v>
       </c>
       <c r="AB20" t="n">
-        <v>-23.3</v>
+        <v>-69.90000000000001</v>
       </c>
       <c r="AC20" t="n">
-        <v>-37.1</v>
+        <v>-111.4</v>
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>(29.2)</t>
+          <t>(87.7)</t>
         </is>
       </c>
       <c r="AE20" t="n">
@@ -2812,14 +2812,14 @@
         <v>0</v>
       </c>
       <c r="AG20" t="n">
-        <v>-31.7</v>
+        <v>-380.8</v>
       </c>
       <c r="AH20" t="n">
-        <v>-29.8</v>
+        <v>-357.3</v>
       </c>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>(26.0)</t>
+          <t>(311.8)</t>
         </is>
       </c>
     </row>
@@ -2936,19 +2936,19 @@
         <v>-18</v>
       </c>
       <c r="AB21" t="n">
-        <v>-21.2</v>
+        <v>-63.7</v>
       </c>
       <c r="AC21" t="n">
-        <v>-16.3</v>
+        <v>-48.9</v>
       </c>
       <c r="AD21" t="n">
-        <v>-28.4</v>
+        <v>-85.3</v>
       </c>
       <c r="AE21" t="n">
-        <v>-19.7</v>
+        <v>-59.2</v>
       </c>
       <c r="AF21" t="n">
-        <v>-22.7</v>
+        <v>-136.5</v>
       </c>
       <c r="AG21" t="n">
         <v>0</v>
@@ -3079,28 +3079,28 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>(20.2)</t>
+          <t>(60.6)</t>
         </is>
       </c>
       <c r="AD22" t="n">
         <v>0</v>
       </c>
       <c r="AE22" t="n">
-        <v>-10</v>
+        <v>-30</v>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>(26.8)</t>
+          <t>(160.6)</t>
         </is>
       </c>
       <c r="AG22" t="n">
         <v>0</v>
       </c>
       <c r="AH22" t="n">
-        <v>-32.8</v>
+        <v>-393.8</v>
       </c>
       <c r="AI22" t="n">
-        <v>-29.5</v>
+        <v>-354.5</v>
       </c>
     </row>
     <row r="23">
@@ -3216,24 +3216,24 @@
         <v>-14.7</v>
       </c>
       <c r="AB23" t="n">
-        <v>-25.2</v>
+        <v>-75.5</v>
       </c>
       <c r="AC23" t="n">
         <v>0</v>
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>(30.5)</t>
+          <t>(91.4)</t>
         </is>
       </c>
       <c r="AE23" t="n">
-        <v>-24.5</v>
+        <v>-73.59999999999999</v>
       </c>
       <c r="AF23" t="n">
         <v>0</v>
       </c>
       <c r="AG23" t="n">
-        <v>-41.3</v>
+        <v>-495.8</v>
       </c>
       <c r="AH23" t="n">
         <v>0</v>
@@ -3356,11 +3356,11 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>(26.4)</t>
+          <t>(79.1)</t>
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>-30.6</v>
+        <v>-91.8</v>
       </c>
       <c r="AD24" t="n">
         <v>0</v>
@@ -3369,11 +3369,11 @@
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>-29.5</v>
+        <v>-176.9</v>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>(25.3)</t>
+          <t>(303.9)</t>
         </is>
       </c>
       <c r="AH24" t="n">
@@ -3496,7 +3496,7 @@
         <v>-12.7</v>
       </c>
       <c r="AB25" t="n">
-        <v>-22.2</v>
+        <v>-66.59999999999999</v>
       </c>
       <c r="AC25" t="n">
         <v>0</v>
@@ -3505,21 +3505,21 @@
         <v>0</v>
       </c>
       <c r="AE25" t="n">
-        <v>-12.2</v>
+        <v>-36.7</v>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>(36.7)</t>
+          <t>(220.1)</t>
         </is>
       </c>
       <c r="AG25" t="n">
         <v>0</v>
       </c>
       <c r="AH25" t="n">
-        <v>-23</v>
+        <v>-276.5</v>
       </c>
       <c r="AI25" t="n">
-        <v>-43.7</v>
+        <v>-524.2</v>
       </c>
     </row>
     <row r="26">
@@ -3639,28 +3639,28 @@
         <v>-28.5</v>
       </c>
       <c r="AB26" t="n">
-        <v>-25.3</v>
+        <v>-75.8</v>
       </c>
       <c r="AC26" t="n">
-        <v>-28.7</v>
+        <v>-86.2</v>
       </c>
       <c r="AD26" t="n">
-        <v>-27.2</v>
+        <v>-81.7</v>
       </c>
       <c r="AE26" t="n">
-        <v>-30.3</v>
+        <v>-91</v>
       </c>
       <c r="AF26" t="n">
         <v>0</v>
       </c>
       <c r="AG26" t="n">
-        <v>-22.5</v>
+        <v>-270.1</v>
       </c>
       <c r="AH26" t="n">
         <v>0</v>
       </c>
       <c r="AI26" t="n">
-        <v>-23.7</v>
+        <v>-284</v>
       </c>
     </row>
     <row r="27">
@@ -3784,24 +3784,24 @@
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>-28.3</v>
+        <v>-85</v>
       </c>
       <c r="AE27" t="n">
-        <v>-21.9</v>
+        <v>-65.59999999999999</v>
       </c>
       <c r="AF27" t="n">
-        <v>-18.3</v>
+        <v>-110</v>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>(10.1)</t>
+          <t>(121.0)</t>
         </is>
       </c>
       <c r="AH27" t="n">
-        <v>-10.2</v>
+        <v>-122</v>
       </c>
       <c r="AI27" t="n">
-        <v>-1.2</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="28">
@@ -3921,27 +3921,27 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>(12.0)</t>
+          <t>(36.0)</t>
         </is>
       </c>
       <c r="AD28" t="n">
-        <v>-7.3</v>
+        <v>-21.8</v>
       </c>
       <c r="AE28" t="n">
         <v>0</v>
       </c>
       <c r="AF28" t="n">
-        <v>-12.4</v>
+        <v>-74.2</v>
       </c>
       <c r="AG28" t="n">
-        <v>-12</v>
+        <v>-143.9</v>
       </c>
       <c r="AH28" t="n">
         <v>0</v>
       </c>
       <c r="AI28" t="inlineStr">
         <is>
-          <t>(12.6)</t>
+          <t>(151.2)</t>
         </is>
       </c>
     </row>
@@ -4062,30 +4062,30 @@
         <v>-54.2</v>
       </c>
       <c r="AB29" t="n">
-        <v>-60.1</v>
+        <v>-180.2</v>
       </c>
       <c r="AC29" t="n">
-        <v>-25</v>
+        <v>-75.09999999999999</v>
       </c>
       <c r="AD29" t="n">
-        <v>-12.5</v>
+        <v>-37.5</v>
       </c>
       <c r="AE29" t="n">
-        <v>-41.8</v>
+        <v>-125.4</v>
       </c>
       <c r="AF29" t="n">
-        <v>-22.6</v>
+        <v>-135.4</v>
       </c>
       <c r="AG29" t="n">
-        <v>-19.4</v>
+        <v>-232.3</v>
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>(31.2)</t>
+          <t>(374.1)</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>-51</v>
+        <v>-611.4</v>
       </c>
     </row>
     <row r="30">
@@ -4218,20 +4218,20 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>-23</v>
+        <v>-69</v>
       </c>
       <c r="AF30" t="n">
-        <v>-17.1</v>
+        <v>-102.5</v>
       </c>
       <c r="AG30" t="n">
-        <v>-14.1</v>
+        <v>-169.5</v>
       </c>
       <c r="AH30" t="n">
-        <v>-13.3</v>
+        <v>-159</v>
       </c>
       <c r="AI30" t="inlineStr">
         <is>
-          <t>(18.7)</t>
+          <t>(223.9)</t>
         </is>
       </c>
     </row>
@@ -4361,24 +4361,24 @@
         <v>0</v>
       </c>
       <c r="AC31" t="n">
-        <v>-40.6</v>
+        <v>-121.7</v>
       </c>
       <c r="AD31" t="n">
-        <v>-23.2</v>
+        <v>-69.5</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
       </c>
       <c r="AF31" t="n">
-        <v>-56.6</v>
+        <v>-339.8</v>
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>(27.2)</t>
+          <t>(326.9)</t>
         </is>
       </c>
       <c r="AH31" t="n">
-        <v>-20.1</v>
+        <v>-241.3</v>
       </c>
       <c r="AI31" t="n">
         <v>0</v>
@@ -4502,31 +4502,31 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>(6.0)</t>
+          <t>(18.1)</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>(15.5)</t>
+          <t>(46.4)</t>
         </is>
       </c>
       <c r="AD32" t="n">
-        <v>-17.8</v>
+        <v>-53.4</v>
       </c>
       <c r="AE32" t="n">
-        <v>-13</v>
+        <v>-39</v>
       </c>
       <c r="AF32" t="n">
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>-8.699999999999999</v>
+        <v>-104</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>-10.7</v>
+        <v>-128.5</v>
       </c>
     </row>
     <row r="33">
@@ -4648,16 +4648,16 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>(20.7)</t>
+          <t>(62.2)</t>
         </is>
       </c>
       <c r="AD33" t="inlineStr">
         <is>
-          <t>(19.4)</t>
+          <t>(58.3)</t>
         </is>
       </c>
       <c r="AE33" t="n">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="AF33" t="n">
         <v>0</v>
@@ -4666,11 +4666,11 @@
         <v>0</v>
       </c>
       <c r="AH33" t="n">
-        <v>-22.5</v>
+        <v>-269.6</v>
       </c>
       <c r="AI33" t="inlineStr">
         <is>
-          <t>(23.5)</t>
+          <t>(282.3)</t>
         </is>
       </c>
     </row>
@@ -4787,13 +4787,13 @@
         <v>37.4</v>
       </c>
       <c r="AB34" t="n">
-        <v>20.7</v>
+        <v>62.1</v>
       </c>
       <c r="AC34" t="n">
         <v>0</v>
       </c>
       <c r="AD34" t="n">
-        <v>37.1</v>
+        <v>111.2</v>
       </c>
       <c r="AE34" t="n">
         <v>0</v>
@@ -4805,10 +4805,10 @@
         <v>0</v>
       </c>
       <c r="AH34" t="n">
-        <v>45</v>
+        <v>539.7</v>
       </c>
       <c r="AI34" t="n">
-        <v>6.1</v>
+        <v>72.59999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -4924,28 +4924,28 @@
         <v>19.6</v>
       </c>
       <c r="AB35" t="n">
-        <v>52.9</v>
+        <v>158.6</v>
       </c>
       <c r="AC35" t="n">
-        <v>46.8</v>
+        <v>140.3</v>
       </c>
       <c r="AD35" t="n">
-        <v>36.2</v>
+        <v>108.6</v>
       </c>
       <c r="AE35" t="n">
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>23.8</v>
+        <v>142.9</v>
       </c>
       <c r="AG35" t="n">
-        <v>55.8</v>
+        <v>669.9</v>
       </c>
       <c r="AH35" t="n">
         <v>0</v>
       </c>
       <c r="AI35" t="n">
-        <v>34.9</v>
+        <v>419.3</v>
       </c>
     </row>
     <row r="36">
@@ -5070,19 +5070,19 @@
         <v>0</v>
       </c>
       <c r="AE36" t="n">
-        <v>0.7</v>
+        <v>2.2</v>
       </c>
       <c r="AF36" t="n">
-        <v>1.6</v>
+        <v>9.5</v>
       </c>
       <c r="AG36" t="n">
         <v>0</v>
       </c>
       <c r="AH36" t="n">
-        <v>2.8</v>
+        <v>33.4</v>
       </c>
       <c r="AI36" t="n">
-        <v>1.9</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="37">
@@ -5198,25 +5198,25 @@
         <v>50.1</v>
       </c>
       <c r="AB37" t="n">
-        <v>54.7</v>
+        <v>164</v>
       </c>
       <c r="AC37" t="n">
-        <v>37.2</v>
+        <v>111.7</v>
       </c>
       <c r="AD37" t="n">
-        <v>35.1</v>
+        <v>105.3</v>
       </c>
       <c r="AE37" t="n">
-        <v>52.6</v>
+        <v>157.9</v>
       </c>
       <c r="AF37" t="n">
         <v>0</v>
       </c>
       <c r="AG37" t="n">
-        <v>44.3</v>
+        <v>531</v>
       </c>
       <c r="AH37" t="n">
-        <v>24.9</v>
+        <v>299.2</v>
       </c>
       <c r="AI37" t="n">
         <v>0</v>
@@ -5335,10 +5335,10 @@
         <v>0</v>
       </c>
       <c r="AB38" t="n">
-        <v>33.6</v>
+        <v>100.9</v>
       </c>
       <c r="AC38" t="n">
-        <v>10.6</v>
+        <v>31.9</v>
       </c>
       <c r="AD38" t="n">
         <v>0</v>
@@ -5350,7 +5350,7 @@
         <v>0</v>
       </c>
       <c r="AG38" t="n">
-        <v>66</v>
+        <v>792</v>
       </c>
       <c r="AH38" t="n">
         <v>0</v>
@@ -5475,19 +5475,19 @@
         <v>0</v>
       </c>
       <c r="AC39" t="n">
-        <v>11.7</v>
+        <v>35</v>
       </c>
       <c r="AD39" t="n">
         <v>0</v>
       </c>
       <c r="AE39" t="n">
-        <v>15.3</v>
+        <v>46</v>
       </c>
       <c r="AF39" t="n">
         <v>0</v>
       </c>
       <c r="AG39" t="n">
-        <v>18</v>
+        <v>216.3</v>
       </c>
       <c r="AH39" t="n">
         <v>0</v>
@@ -5609,28 +5609,28 @@
         <v>4.5</v>
       </c>
       <c r="AB40" t="n">
-        <v>7.3</v>
+        <v>21.9</v>
       </c>
       <c r="AC40" t="n">
         <v>0</v>
       </c>
       <c r="AD40" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AE40" t="n">
-        <v>5.6</v>
+        <v>16.7</v>
       </c>
       <c r="AF40" t="n">
         <v>0</v>
       </c>
       <c r="AG40" t="n">
-        <v>6.8</v>
+        <v>81.2</v>
       </c>
       <c r="AH40" t="n">
-        <v>6.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AI40" t="n">
-        <v>5.2</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="41">
@@ -5746,16 +5746,16 @@
         <v>30.1</v>
       </c>
       <c r="AB41" t="n">
-        <v>18.5</v>
+        <v>55.6</v>
       </c>
       <c r="AC41" t="n">
-        <v>28.4</v>
+        <v>85.2</v>
       </c>
       <c r="AD41" t="n">
-        <v>3.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AE41" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="AF41" t="n">
         <v>0</v>
@@ -5767,7 +5767,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="n">
-        <v>20.4</v>
+        <v>244.7</v>
       </c>
     </row>
     <row r="42">
@@ -5883,28 +5883,28 @@
         <v>22.4</v>
       </c>
       <c r="AB42" t="n">
-        <v>24.8</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="AC42" t="n">
-        <v>35.4</v>
+        <v>106.3</v>
       </c>
       <c r="AD42" t="n">
-        <v>22.9</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AE42" t="n">
         <v>0</v>
       </c>
       <c r="AF42" t="n">
-        <v>12.5</v>
+        <v>75</v>
       </c>
       <c r="AG42" t="n">
-        <v>15.4</v>
+        <v>185</v>
       </c>
       <c r="AH42" t="n">
-        <v>15.5</v>
+        <v>186.4</v>
       </c>
       <c r="AI42" t="n">
-        <v>28.7</v>
+        <v>344.6</v>
       </c>
     </row>
     <row r="43">
@@ -6020,28 +6020,28 @@
         <v>36.9</v>
       </c>
       <c r="AB43" t="n">
-        <v>10</v>
+        <v>29.9</v>
       </c>
       <c r="AC43" t="n">
-        <v>36.5</v>
+        <v>109.4</v>
       </c>
       <c r="AD43" t="n">
-        <v>8.5</v>
+        <v>25.6</v>
       </c>
       <c r="AE43" t="n">
-        <v>52.4</v>
+        <v>157.2</v>
       </c>
       <c r="AF43" t="n">
-        <v>46.3</v>
+        <v>277.6</v>
       </c>
       <c r="AG43" t="n">
-        <v>29.2</v>
+        <v>350.3</v>
       </c>
       <c r="AH43" t="n">
         <v>0</v>
       </c>
       <c r="AI43" t="n">
-        <v>54.9</v>
+        <v>659.4</v>
       </c>
     </row>
     <row r="44">
@@ -6157,28 +6157,28 @@
         <v>13.4</v>
       </c>
       <c r="AB44" t="n">
-        <v>23.8</v>
+        <v>71.3</v>
       </c>
       <c r="AC44" t="n">
-        <v>16.6</v>
+        <v>49.8</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.6</v>
+        <v>1.9</v>
       </c>
       <c r="AE44" t="n">
         <v>0</v>
       </c>
       <c r="AF44" t="n">
-        <v>12.5</v>
+        <v>74.8</v>
       </c>
       <c r="AG44" t="n">
-        <v>16.2</v>
+        <v>194.7</v>
       </c>
       <c r="AH44" t="n">
-        <v>13.1</v>
+        <v>156.7</v>
       </c>
       <c r="AI44" t="n">
-        <v>20.6</v>
+        <v>246.9</v>
       </c>
     </row>
     <row r="45">
@@ -6294,28 +6294,28 @@
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>23.9</v>
+        <v>71.7</v>
       </c>
       <c r="AC45" t="n">
-        <v>16.9</v>
+        <v>50.6</v>
       </c>
       <c r="AD45" t="n">
-        <v>22.4</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AE45" t="n">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="AF45" t="n">
-        <v>25.6</v>
+        <v>153.8</v>
       </c>
       <c r="AG45" t="n">
-        <v>28.3</v>
+        <v>339.1</v>
       </c>
       <c r="AH45" t="n">
-        <v>15.8</v>
+        <v>189.1</v>
       </c>
       <c r="AI45" t="n">
-        <v>20</v>
+        <v>240.5</v>
       </c>
     </row>
     <row r="46">
@@ -6431,7 +6431,7 @@
         <v>20.8</v>
       </c>
       <c r="AB46" t="n">
-        <v>45.3</v>
+        <v>136</v>
       </c>
       <c r="AC46" t="n">
         <v>0</v>
@@ -6440,19 +6440,19 @@
         <v>0</v>
       </c>
       <c r="AE46" t="n">
-        <v>57.8</v>
+        <v>173.5</v>
       </c>
       <c r="AF46" t="n">
-        <v>48.7</v>
+        <v>292.4</v>
       </c>
       <c r="AG46" t="n">
-        <v>41.2</v>
+        <v>494.3</v>
       </c>
       <c r="AH46" t="n">
-        <v>68.2</v>
+        <v>818.3</v>
       </c>
       <c r="AI46" t="n">
-        <v>6.8</v>
+        <v>82</v>
       </c>
     </row>
     <row r="47">
@@ -6571,19 +6571,19 @@
         <v>0</v>
       </c>
       <c r="AC47" t="n">
-        <v>3.8</v>
+        <v>11.4</v>
       </c>
       <c r="AD47" t="n">
-        <v>9.4</v>
+        <v>28.3</v>
       </c>
       <c r="AE47" t="n">
-        <v>7.2</v>
+        <v>21.5</v>
       </c>
       <c r="AF47" t="n">
-        <v>6.2</v>
+        <v>37.5</v>
       </c>
       <c r="AG47" t="n">
-        <v>10.6</v>
+        <v>127.5</v>
       </c>
       <c r="AH47" t="n">
         <v>0</v>
@@ -6708,25 +6708,25 @@
         <v>0</v>
       </c>
       <c r="AC48" t="n">
-        <v>29</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="AD48" t="n">
         <v>0</v>
       </c>
       <c r="AE48" t="n">
-        <v>15.8</v>
+        <v>47.3</v>
       </c>
       <c r="AF48" t="n">
-        <v>33.9</v>
+        <v>203.2</v>
       </c>
       <c r="AG48" t="n">
-        <v>26.1</v>
+        <v>313.7</v>
       </c>
       <c r="AH48" t="n">
-        <v>16.1</v>
+        <v>193.4</v>
       </c>
       <c r="AI48" t="n">
-        <v>16.5</v>
+        <v>198.5</v>
       </c>
     </row>
     <row r="49">
@@ -6842,28 +6842,28 @@
         <v>17.9</v>
       </c>
       <c r="AB49" t="n">
-        <v>10.8</v>
+        <v>32.3</v>
       </c>
       <c r="AC49" t="n">
-        <v>5</v>
+        <v>14.9</v>
       </c>
       <c r="AD49" t="n">
-        <v>13</v>
+        <v>38.9</v>
       </c>
       <c r="AE49" t="n">
-        <v>11.6</v>
+        <v>34.9</v>
       </c>
       <c r="AF49" t="n">
-        <v>8.5</v>
+        <v>51.1</v>
       </c>
       <c r="AG49" t="n">
-        <v>16.1</v>
+        <v>192.7</v>
       </c>
       <c r="AH49" t="n">
-        <v>2</v>
+        <v>23.5</v>
       </c>
       <c r="AI49" t="n">
-        <v>4.1</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="50">
@@ -6982,25 +6982,25 @@
         <v>0</v>
       </c>
       <c r="AC50" t="n">
-        <v>8.9</v>
+        <v>26.6</v>
       </c>
       <c r="AD50" t="n">
-        <v>16.9</v>
+        <v>50.8</v>
       </c>
       <c r="AE50" t="n">
-        <v>13.1</v>
+        <v>39.4</v>
       </c>
       <c r="AF50" t="n">
         <v>0</v>
       </c>
       <c r="AG50" t="n">
-        <v>29.5</v>
+        <v>354.4</v>
       </c>
       <c r="AH50" t="n">
         <v>0</v>
       </c>
       <c r="AI50" t="n">
-        <v>11.6</v>
+        <v>139.7</v>
       </c>
     </row>
     <row r="51">
@@ -7126,23 +7126,23 @@
         <v>-20.4</v>
       </c>
       <c r="AB51" t="n">
-        <v>-26.8</v>
+        <v>-80.5</v>
       </c>
       <c r="AC51" t="n">
-        <v>-22.2</v>
+        <v>-66.5</v>
       </c>
       <c r="AD51" t="n">
         <v>0</v>
       </c>
       <c r="AE51" t="n">
-        <v>-26</v>
+        <v>-77.90000000000001</v>
       </c>
       <c r="AF51" t="n">
-        <v>-22.6</v>
+        <v>-135.4</v>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>(30.5)</t>
+          <t>(365.9)</t>
         </is>
       </c>
       <c r="AH51" t="n">
@@ -7265,24 +7265,24 @@
         <v>0</v>
       </c>
       <c r="AB52" t="n">
-        <v>-13.1</v>
+        <v>-39.2</v>
       </c>
       <c r="AC52" t="inlineStr">
         <is>
-          <t>(13.9)</t>
+          <t>(41.6)</t>
         </is>
       </c>
       <c r="AD52" t="n">
-        <v>-18.9</v>
+        <v>-56.8</v>
       </c>
       <c r="AE52" t="n">
-        <v>-12.5</v>
+        <v>-37.6</v>
       </c>
       <c r="AF52" t="n">
-        <v>-9.800000000000001</v>
+        <v>-58.5</v>
       </c>
       <c r="AG52" t="n">
-        <v>-11.3</v>
+        <v>-135.1</v>
       </c>
       <c r="AH52" t="n">
         <v>0</v>
@@ -7410,30 +7410,30 @@
         </is>
       </c>
       <c r="AB53" t="n">
-        <v>-4.4</v>
+        <v>-13.1</v>
       </c>
       <c r="AC53" t="n">
-        <v>-14.3</v>
+        <v>-43</v>
       </c>
       <c r="AD53" t="n">
         <v>0</v>
       </c>
       <c r="AE53" t="inlineStr">
         <is>
-          <t>(11.4)</t>
+          <t>(34.1)</t>
         </is>
       </c>
       <c r="AF53" t="n">
-        <v>-9.800000000000001</v>
+        <v>-58.6</v>
       </c>
       <c r="AG53" t="n">
-        <v>-13.3</v>
+        <v>-159.5</v>
       </c>
       <c r="AH53" t="n">
-        <v>-13</v>
+        <v>-156.6</v>
       </c>
       <c r="AI53" t="n">
-        <v>-12.7</v>
+        <v>-152.3</v>
       </c>
     </row>
     <row r="54">
@@ -7551,7 +7551,7 @@
         <v>-5.3</v>
       </c>
       <c r="AB54" t="n">
-        <v>-4.2</v>
+        <v>-12.6</v>
       </c>
       <c r="AC54" t="n">
         <v>0</v>
@@ -7560,20 +7560,20 @@
         <v>0</v>
       </c>
       <c r="AE54" t="n">
-        <v>-3.2</v>
+        <v>-9.5</v>
       </c>
       <c r="AF54" t="n">
-        <v>-8.4</v>
+        <v>-50.3</v>
       </c>
       <c r="AG54" t="n">
-        <v>-8</v>
+        <v>-95.7</v>
       </c>
       <c r="AH54" t="n">
         <v>0</v>
       </c>
       <c r="AI54" t="inlineStr">
         <is>
-          <t>(4.4)</t>
+          <t>(53.2)</t>
         </is>
       </c>
     </row>
@@ -7698,13 +7698,13 @@
         <v>0</v>
       </c>
       <c r="AD55" t="n">
-        <v>-33.8</v>
+        <v>-101.4</v>
       </c>
       <c r="AE55" t="n">
         <v>0</v>
       </c>
       <c r="AF55" t="n">
-        <v>-45.4</v>
+        <v>-272.3</v>
       </c>
       <c r="AG55" t="n">
         <v>0</v>
@@ -7713,7 +7713,7 @@
         <v>0</v>
       </c>
       <c r="AI55" t="n">
-        <v>-39.7</v>
+        <v>-476.4</v>
       </c>
     </row>
     <row r="56">
@@ -7836,32 +7836,32 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>(17.5)</t>
+          <t>(52.4)</t>
         </is>
       </c>
       <c r="AC56" t="inlineStr">
         <is>
-          <t>(43.5)</t>
+          <t>(130.4)</t>
         </is>
       </c>
       <c r="AD56" t="n">
         <v>0</v>
       </c>
       <c r="AE56" t="n">
-        <v>-39.7</v>
+        <v>-119.2</v>
       </c>
       <c r="AF56" t="n">
-        <v>-23.1</v>
+        <v>-138.9</v>
       </c>
       <c r="AG56" t="n">
         <v>0</v>
       </c>
       <c r="AH56" t="n">
-        <v>-29.6</v>
+        <v>-355.3</v>
       </c>
       <c r="AI56" t="inlineStr">
         <is>
-          <t>(35.9)</t>
+          <t>(430.5)</t>
         </is>
       </c>
     </row>
@@ -7981,14 +7981,14 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>(18.7)</t>
+          <t>(56.2)</t>
         </is>
       </c>
       <c r="AC57" t="n">
-        <v>-16.9</v>
+        <v>-50.6</v>
       </c>
       <c r="AD57" t="n">
-        <v>-7.1</v>
+        <v>-21.3</v>
       </c>
       <c r="AE57" t="n">
         <v>0</v>
@@ -7997,10 +7997,10 @@
         <v>0</v>
       </c>
       <c r="AG57" t="n">
-        <v>-11.7</v>
+        <v>-140</v>
       </c>
       <c r="AH57" t="n">
-        <v>-12</v>
+        <v>-144.6</v>
       </c>
       <c r="AI57" t="n">
         <v>0</v>
@@ -8128,29 +8128,29 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>(4.2)</t>
+          <t>(12.5)</t>
         </is>
       </c>
       <c r="AC58" t="n">
         <v>0</v>
       </c>
       <c r="AD58" t="n">
-        <v>-15.5</v>
+        <v>-46.6</v>
       </c>
       <c r="AE58" t="n">
-        <v>-11</v>
+        <v>-32.9</v>
       </c>
       <c r="AF58" t="n">
-        <v>-16.5</v>
+        <v>-98.7</v>
       </c>
       <c r="AG58" t="n">
-        <v>-17.2</v>
+        <v>-206.3</v>
       </c>
       <c r="AH58" t="n">
-        <v>-9.800000000000001</v>
+        <v>-118.1</v>
       </c>
       <c r="AI58" t="n">
-        <v>-17.1</v>
+        <v>-205.1</v>
       </c>
     </row>
     <row r="59">
@@ -8269,17 +8269,17 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>(17.6)</t>
+          <t>(52.8)</t>
         </is>
       </c>
       <c r="AC59" t="n">
         <v>0</v>
       </c>
       <c r="AD59" t="n">
-        <v>-7.9</v>
+        <v>-23.7</v>
       </c>
       <c r="AE59" t="n">
-        <v>-13.8</v>
+        <v>-41.3</v>
       </c>
       <c r="AF59" t="n">
         <v>0</v>
@@ -8291,7 +8291,7 @@
         <v>0</v>
       </c>
       <c r="AI59" t="n">
-        <v>-16.8</v>
+        <v>-201.6</v>
       </c>
     </row>
     <row r="60">
@@ -8418,23 +8418,23 @@
       </c>
       <c r="AD60" t="inlineStr">
         <is>
-          <t>(23.2)</t>
+          <t>(69.7)</t>
         </is>
       </c>
       <c r="AE60" t="n">
         <v>0</v>
       </c>
       <c r="AF60" t="n">
-        <v>-16</v>
+        <v>-96.09999999999999</v>
       </c>
       <c r="AG60" t="n">
-        <v>-30.8</v>
+        <v>-370.1</v>
       </c>
       <c r="AH60" t="n">
-        <v>-14.8</v>
+        <v>-177.1</v>
       </c>
       <c r="AI60" t="n">
-        <v>-18.5</v>
+        <v>-221.8</v>
       </c>
     </row>
     <row r="61">
@@ -8554,30 +8554,30 @@
         <v>-14.1</v>
       </c>
       <c r="AB61" t="n">
-        <v>-12.6</v>
+        <v>-37.9</v>
       </c>
       <c r="AC61" t="n">
         <v>0</v>
       </c>
       <c r="AD61" t="inlineStr">
         <is>
-          <t>(16.3)</t>
+          <t>(49.0)</t>
         </is>
       </c>
       <c r="AE61" t="n">
-        <v>-13.8</v>
+        <v>-41.3</v>
       </c>
       <c r="AF61" t="n">
         <v>0</v>
       </c>
       <c r="AG61" t="n">
-        <v>-5.8</v>
+        <v>-70.09999999999999</v>
       </c>
       <c r="AH61" t="n">
-        <v>-10</v>
+        <v>-119.9</v>
       </c>
       <c r="AI61" t="n">
-        <v>-8.1</v>
+        <v>-97.7</v>
       </c>
     </row>
     <row r="62">
@@ -8697,22 +8697,22 @@
         <v>-10.8</v>
       </c>
       <c r="AB62" t="n">
-        <v>-13.6</v>
+        <v>-40.7</v>
       </c>
       <c r="AC62" t="n">
         <v>0</v>
       </c>
       <c r="AD62" t="n">
-        <v>-15.2</v>
+        <v>-45.5</v>
       </c>
       <c r="AE62" t="n">
-        <v>-11.2</v>
+        <v>-33.5</v>
       </c>
       <c r="AF62" t="n">
-        <v>-13.3</v>
+        <v>-79.8</v>
       </c>
       <c r="AG62" t="n">
-        <v>-6.9</v>
+        <v>-83.3</v>
       </c>
       <c r="AH62" t="n">
         <v>0</v>
@@ -8835,29 +8835,29 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>(12.6)</t>
+          <t>(37.7)</t>
         </is>
       </c>
       <c r="AC63" t="n">
         <v>0</v>
       </c>
       <c r="AD63" t="n">
-        <v>-0.4</v>
+        <v>-1.1</v>
       </c>
       <c r="AE63" t="n">
-        <v>-8.300000000000001</v>
+        <v>-24.9</v>
       </c>
       <c r="AF63" t="n">
         <v>0</v>
       </c>
       <c r="AG63" t="n">
-        <v>-11.9</v>
+        <v>-142.5</v>
       </c>
       <c r="AH63" t="n">
-        <v>-9.4</v>
+        <v>-112.9</v>
       </c>
       <c r="AI63" t="n">
-        <v>-4</v>
+        <v>-48</v>
       </c>
     </row>
     <row r="64">
@@ -8978,14 +8978,14 @@
         <v>0</v>
       </c>
       <c r="AC64" t="n">
-        <v>-9</v>
+        <v>-27.1</v>
       </c>
       <c r="AD64" t="n">
-        <v>-15.6</v>
+        <v>-46.9</v>
       </c>
       <c r="AE64" t="inlineStr">
         <is>
-          <t>(35.4)</t>
+          <t>(106.3)</t>
         </is>
       </c>
       <c r="AF64" t="n">
@@ -8993,14 +8993,14 @@
       </c>
       <c r="AG64" t="inlineStr">
         <is>
-          <t>(26.1)</t>
+          <t>(313.3)</t>
         </is>
       </c>
       <c r="AH64" t="n">
         <v>0</v>
       </c>
       <c r="AI64" t="n">
-        <v>-18</v>
+        <v>-216.1</v>
       </c>
     </row>
     <row r="65">
@@ -9118,29 +9118,29 @@
         <v>-19.6</v>
       </c>
       <c r="AB65" t="n">
-        <v>-13.3</v>
+        <v>-39.9</v>
       </c>
       <c r="AC65" t="inlineStr">
         <is>
-          <t>(9.3)</t>
+          <t>(27.9)</t>
         </is>
       </c>
       <c r="AD65" t="n">
-        <v>-24.6</v>
+        <v>-73.8</v>
       </c>
       <c r="AE65" t="inlineStr">
         <is>
-          <t>(13.1)</t>
+          <t>(39.3)</t>
         </is>
       </c>
       <c r="AF65" t="n">
-        <v>-30.5</v>
+        <v>-183.3</v>
       </c>
       <c r="AG65" t="n">
         <v>0</v>
       </c>
       <c r="AH65" t="n">
-        <v>-21.4</v>
+        <v>-257.3</v>
       </c>
       <c r="AI65" t="n">
         <v>0</v>
@@ -9259,33 +9259,33 @@
         <v>-2.7</v>
       </c>
       <c r="AB66" t="n">
-        <v>-3.7</v>
+        <v>-11.1</v>
       </c>
       <c r="AC66" t="n">
-        <v>-0.3</v>
+        <v>-1</v>
       </c>
       <c r="AD66" t="inlineStr">
         <is>
-          <t>(1.9)</t>
+          <t>(5.8)</t>
         </is>
       </c>
       <c r="AE66" t="n">
-        <v>-2.6</v>
+        <v>-7.8</v>
       </c>
       <c r="AF66" t="n">
-        <v>-1.4</v>
+        <v>-8.6</v>
       </c>
       <c r="AG66" t="n">
-        <v>-3</v>
+        <v>-36.5</v>
       </c>
       <c r="AH66" t="inlineStr">
         <is>
-          <t>(3.3)</t>
+          <t>(39.2)</t>
         </is>
       </c>
       <c r="AI66" t="inlineStr">
         <is>
-          <t>(5.5)</t>
+          <t>(65.9)</t>
         </is>
       </c>
     </row>
@@ -9405,25 +9405,25 @@
         <v>0</v>
       </c>
       <c r="AC67" t="n">
-        <v>7.5</v>
+        <v>22.6</v>
       </c>
       <c r="AD67" t="n">
         <v>0</v>
       </c>
       <c r="AE67" t="n">
-        <v>22.9</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AF67" t="n">
-        <v>40.6</v>
+        <v>243.7</v>
       </c>
       <c r="AG67" t="n">
-        <v>45.3</v>
+        <v>543.3</v>
       </c>
       <c r="AH67" t="n">
         <v>0</v>
       </c>
       <c r="AI67" t="n">
-        <v>20.7</v>
+        <v>248.7</v>
       </c>
     </row>
     <row r="68">
@@ -9542,7 +9542,7 @@
         <v>0</v>
       </c>
       <c r="AC68" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AD68" t="n">
         <v>0</v>
@@ -9551,16 +9551,16 @@
         <v>0</v>
       </c>
       <c r="AF68" t="n">
-        <v>8.300000000000001</v>
+        <v>49.9</v>
       </c>
       <c r="AG68" t="n">
-        <v>6.3</v>
+        <v>75.5</v>
       </c>
       <c r="AH68" t="n">
         <v>0</v>
       </c>
       <c r="AI68" t="n">
-        <v>7.2</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="69">
@@ -9676,28 +9676,28 @@
         <v>6.4</v>
       </c>
       <c r="AB69" t="n">
-        <v>11.3</v>
+        <v>33.9</v>
       </c>
       <c r="AC69" t="n">
-        <v>12.6</v>
+        <v>37.7</v>
       </c>
       <c r="AD69" t="n">
-        <v>13.4</v>
+        <v>40.3</v>
       </c>
       <c r="AE69" t="n">
         <v>0</v>
       </c>
       <c r="AF69" t="n">
-        <v>9.4</v>
+        <v>56.6</v>
       </c>
       <c r="AG69" t="n">
         <v>0</v>
       </c>
       <c r="AH69" t="n">
-        <v>9.6</v>
+        <v>115.3</v>
       </c>
       <c r="AI69" t="n">
-        <v>9.300000000000001</v>
+        <v>111.8</v>
       </c>
     </row>
     <row r="70">
@@ -9813,28 +9813,28 @@
         <v>16.4</v>
       </c>
       <c r="AB70" t="n">
-        <v>15.9</v>
+        <v>47.8</v>
       </c>
       <c r="AC70" t="n">
-        <v>7.1</v>
+        <v>21.2</v>
       </c>
       <c r="AD70" t="n">
-        <v>23.7</v>
+        <v>71.2</v>
       </c>
       <c r="AE70" t="n">
-        <v>22.6</v>
+        <v>67.8</v>
       </c>
       <c r="AF70" t="n">
-        <v>26.1</v>
+        <v>156.9</v>
       </c>
       <c r="AG70" t="n">
-        <v>20.4</v>
+        <v>245</v>
       </c>
       <c r="AH70" t="n">
-        <v>26.7</v>
+        <v>320.5</v>
       </c>
       <c r="AI70" t="n">
-        <v>9.4</v>
+        <v>112.6</v>
       </c>
     </row>
     <row r="71">
@@ -9959,19 +9959,19 @@
         <v>0</v>
       </c>
       <c r="AE71" t="n">
-        <v>35.7</v>
+        <v>107</v>
       </c>
       <c r="AF71" t="n">
         <v>0</v>
       </c>
       <c r="AG71" t="n">
-        <v>24.2</v>
+        <v>290</v>
       </c>
       <c r="AH71" t="n">
         <v>0</v>
       </c>
       <c r="AI71" t="n">
-        <v>7.9</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="72">
@@ -10087,28 +10087,28 @@
         <v>25.3</v>
       </c>
       <c r="AB72" t="n">
-        <v>14.7</v>
+        <v>44.2</v>
       </c>
       <c r="AC72" t="n">
-        <v>14.4</v>
+        <v>43.3</v>
       </c>
       <c r="AD72" t="n">
         <v>0</v>
       </c>
       <c r="AE72" t="n">
-        <v>8.699999999999999</v>
+        <v>26</v>
       </c>
       <c r="AF72" t="n">
-        <v>14</v>
+        <v>83.7</v>
       </c>
       <c r="AG72" t="n">
         <v>0</v>
       </c>
       <c r="AH72" t="n">
-        <v>15.5</v>
+        <v>186.5</v>
       </c>
       <c r="AI72" t="n">
-        <v>14.2</v>
+        <v>170.3</v>
       </c>
     </row>
     <row r="73">
@@ -10236,16 +10236,16 @@
         <v>0</v>
       </c>
       <c r="AF73" t="n">
-        <v>45.4</v>
+        <v>272.4</v>
       </c>
       <c r="AG73" t="n">
-        <v>40.6</v>
+        <v>486.7</v>
       </c>
       <c r="AH73" t="n">
-        <v>39</v>
+        <v>468.2</v>
       </c>
       <c r="AI73" t="n">
-        <v>40.2</v>
+        <v>482.1</v>
       </c>
     </row>
     <row r="74">
@@ -10361,22 +10361,22 @@
         <v>15.5</v>
       </c>
       <c r="AB74" t="n">
-        <v>8.9</v>
+        <v>26.6</v>
       </c>
       <c r="AC74" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="AD74" t="n">
         <v>0</v>
       </c>
       <c r="AE74" t="n">
-        <v>6.4</v>
+        <v>19.1</v>
       </c>
       <c r="AF74" t="n">
-        <v>4.8</v>
+        <v>28.6</v>
       </c>
       <c r="AG74" t="n">
-        <v>12.3</v>
+        <v>147.1</v>
       </c>
       <c r="AH74" t="n">
         <v>0</v>
@@ -10498,25 +10498,25 @@
         <v>0</v>
       </c>
       <c r="AB75" t="n">
-        <v>24.3</v>
+        <v>73</v>
       </c>
       <c r="AC75" t="n">
-        <v>27.7</v>
+        <v>83.2</v>
       </c>
       <c r="AD75" t="n">
         <v>0</v>
       </c>
       <c r="AE75" t="n">
-        <v>28.3</v>
+        <v>84.8</v>
       </c>
       <c r="AF75" t="n">
-        <v>40.8</v>
+        <v>244.6</v>
       </c>
       <c r="AG75" t="n">
         <v>0</v>
       </c>
       <c r="AH75" t="n">
-        <v>52.5</v>
+        <v>629.8</v>
       </c>
       <c r="AI75" t="n">
         <v>0</v>
@@ -10635,25 +10635,25 @@
         <v>24.3</v>
       </c>
       <c r="AB76" t="n">
-        <v>6.3</v>
+        <v>18.8</v>
       </c>
       <c r="AC76" t="n">
-        <v>23.4</v>
+        <v>70.2</v>
       </c>
       <c r="AD76" t="n">
-        <v>38.3</v>
+        <v>115</v>
       </c>
       <c r="AE76" t="n">
-        <v>11.4</v>
+        <v>34.3</v>
       </c>
       <c r="AF76" t="n">
         <v>0</v>
       </c>
       <c r="AG76" t="n">
-        <v>32</v>
+        <v>383.9</v>
       </c>
       <c r="AH76" t="n">
-        <v>32.6</v>
+        <v>390.9</v>
       </c>
       <c r="AI76" t="n">
         <v>0</v>
@@ -10778,22 +10778,22 @@
         <v>0</v>
       </c>
       <c r="AD77" t="n">
-        <v>11.2</v>
+        <v>33.6</v>
       </c>
       <c r="AE77" t="n">
         <v>0</v>
       </c>
       <c r="AF77" t="n">
-        <v>9.5</v>
+        <v>57</v>
       </c>
       <c r="AG77" t="n">
         <v>0</v>
       </c>
       <c r="AH77" t="n">
-        <v>5.5</v>
+        <v>65.7</v>
       </c>
       <c r="AI77" t="n">
-        <v>11.2</v>
+        <v>134.8</v>
       </c>
     </row>
     <row r="78">
@@ -10909,25 +10909,25 @@
         <v>33.2</v>
       </c>
       <c r="AB78" t="n">
-        <v>39.3</v>
+        <v>117.8</v>
       </c>
       <c r="AC78" t="n">
-        <v>21.6</v>
+        <v>64.7</v>
       </c>
       <c r="AD78" t="n">
-        <v>22</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="AE78" t="n">
-        <v>44.1</v>
+        <v>132.4</v>
       </c>
       <c r="AF78" t="n">
-        <v>48.1</v>
+        <v>288.5</v>
       </c>
       <c r="AG78" t="n">
         <v>0</v>
       </c>
       <c r="AH78" t="n">
-        <v>38.7</v>
+        <v>464.2</v>
       </c>
       <c r="AI78" t="n">
         <v>0</v>
@@ -11046,13 +11046,13 @@
         <v>0</v>
       </c>
       <c r="AB79" t="n">
-        <v>26.6</v>
+        <v>79.7</v>
       </c>
       <c r="AC79" t="n">
-        <v>26.2</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="AD79" t="n">
-        <v>38.5</v>
+        <v>115.6</v>
       </c>
       <c r="AE79" t="n">
         <v>0</v>
@@ -11061,10 +11061,10 @@
         <v>0</v>
       </c>
       <c r="AG79" t="n">
-        <v>14.4</v>
+        <v>172.2</v>
       </c>
       <c r="AH79" t="n">
-        <v>17.6</v>
+        <v>211</v>
       </c>
       <c r="AI79" t="n">
         <v>0</v>
@@ -11183,28 +11183,28 @@
         <v>1.8</v>
       </c>
       <c r="AB80" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AC80" t="n">
-        <v>4.4</v>
+        <v>13.1</v>
       </c>
       <c r="AD80" t="n">
         <v>0</v>
       </c>
       <c r="AE80" t="n">
-        <v>4.3</v>
+        <v>13</v>
       </c>
       <c r="AF80" t="n">
-        <v>3</v>
+        <v>17.8</v>
       </c>
       <c r="AG80" t="n">
-        <v>2.7</v>
+        <v>32.5</v>
       </c>
       <c r="AH80" t="n">
         <v>0</v>
       </c>
       <c r="AI80" t="n">
-        <v>3.2</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="81">
@@ -11320,10 +11320,10 @@
         <v>0</v>
       </c>
       <c r="AB81" t="n">
-        <v>31.6</v>
+        <v>94.8</v>
       </c>
       <c r="AC81" t="n">
-        <v>20.4</v>
+        <v>61.2</v>
       </c>
       <c r="AD81" t="n">
         <v>0</v>
@@ -11332,13 +11332,13 @@
         <v>0</v>
       </c>
       <c r="AF81" t="n">
-        <v>27.5</v>
+        <v>164.9</v>
       </c>
       <c r="AG81" t="n">
         <v>0</v>
       </c>
       <c r="AH81" t="n">
-        <v>21.8</v>
+        <v>261.1</v>
       </c>
       <c r="AI81" t="n">
         <v>0</v>
@@ -11457,19 +11457,19 @@
         <v>16.1</v>
       </c>
       <c r="AB82" t="n">
-        <v>6.3</v>
+        <v>18.8</v>
       </c>
       <c r="AC82" t="n">
-        <v>25.1</v>
+        <v>75.2</v>
       </c>
       <c r="AD82" t="n">
-        <v>22.3</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AE82" t="n">
         <v>0</v>
       </c>
       <c r="AF82" t="n">
-        <v>22.4</v>
+        <v>134.3</v>
       </c>
       <c r="AG82" t="n">
         <v>0</v>
@@ -11478,7 +11478,7 @@
         <v>0</v>
       </c>
       <c r="AI82" t="n">
-        <v>24.9</v>
+        <v>299.3</v>
       </c>
     </row>
     <row r="83">
@@ -11594,25 +11594,25 @@
         <v>30.3</v>
       </c>
       <c r="AB83" t="n">
-        <v>21</v>
+        <v>63.1</v>
       </c>
       <c r="AC83" t="n">
-        <v>42</v>
+        <v>126</v>
       </c>
       <c r="AD83" t="n">
         <v>0</v>
       </c>
       <c r="AE83" t="n">
-        <v>22.3</v>
+        <v>67</v>
       </c>
       <c r="AF83" t="n">
-        <v>60.2</v>
+        <v>361.4</v>
       </c>
       <c r="AG83" t="n">
         <v>0</v>
       </c>
       <c r="AH83" t="n">
-        <v>60.9</v>
+        <v>730.8</v>
       </c>
       <c r="AI83" t="n">
         <v>0</v>
@@ -11734,7 +11734,7 @@
         <v>0</v>
       </c>
       <c r="AC84" t="n">
-        <v>43.1</v>
+        <v>129.2</v>
       </c>
       <c r="AD84" t="n">
         <v>0</v>
@@ -11749,10 +11749,10 @@
         <v>0</v>
       </c>
       <c r="AH84" t="n">
-        <v>4.4</v>
+        <v>53.3</v>
       </c>
       <c r="AI84" t="n">
-        <v>24.6</v>
+        <v>295.2</v>
       </c>
     </row>
     <row r="85">
@@ -11868,16 +11868,16 @@
         <v>10.9</v>
       </c>
       <c r="AB85" t="n">
-        <v>9.5</v>
+        <v>28.6</v>
       </c>
       <c r="AC85" t="n">
-        <v>9.6</v>
+        <v>28.7</v>
       </c>
       <c r="AD85" t="n">
-        <v>12.5</v>
+        <v>37.5</v>
       </c>
       <c r="AE85" t="n">
-        <v>8.5</v>
+        <v>25.5</v>
       </c>
       <c r="AF85" t="n">
         <v>0</v>
@@ -11886,7 +11886,7 @@
         <v>0</v>
       </c>
       <c r="AH85" t="n">
-        <v>12.2</v>
+        <v>145.9</v>
       </c>
       <c r="AI85" t="n">
         <v>0</v>
@@ -12008,16 +12008,16 @@
         <v>0</v>
       </c>
       <c r="AC86" t="n">
-        <v>9.1</v>
+        <v>27.2</v>
       </c>
       <c r="AD86" t="n">
-        <v>40.5</v>
+        <v>121.5</v>
       </c>
       <c r="AE86" t="n">
         <v>0</v>
       </c>
       <c r="AF86" t="n">
-        <v>41.9</v>
+        <v>251.6</v>
       </c>
       <c r="AG86" t="n">
         <v>0</v>
@@ -12157,13 +12157,13 @@
         <v>0</v>
       </c>
       <c r="AG87" t="n">
-        <v>38.6</v>
+        <v>462.6</v>
       </c>
       <c r="AH87" t="n">
         <v>0</v>
       </c>
       <c r="AI87" t="n">
-        <v>27.3</v>
+        <v>327.7</v>
       </c>
     </row>
     <row r="88">
@@ -12279,28 +12279,28 @@
         <v>1.2</v>
       </c>
       <c r="AB88" t="n">
-        <v>1.2</v>
+        <v>3.7</v>
       </c>
       <c r="AC88" t="n">
         <v>0</v>
       </c>
       <c r="AD88" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="AE88" t="n">
         <v>0</v>
       </c>
       <c r="AF88" t="n">
-        <v>3.3</v>
+        <v>19.6</v>
       </c>
       <c r="AG88" t="n">
         <v>0</v>
       </c>
       <c r="AH88" t="n">
-        <v>0.7</v>
+        <v>8.1</v>
       </c>
       <c r="AI88" t="n">
-        <v>2</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="89">
@@ -12416,28 +12416,28 @@
         <v>0</v>
       </c>
       <c r="AB89" t="n">
-        <v>1.7</v>
+        <v>5</v>
       </c>
       <c r="AC89" t="n">
         <v>0</v>
       </c>
       <c r="AD89" t="n">
-        <v>0.8</v>
+        <v>2.4</v>
       </c>
       <c r="AE89" t="n">
-        <v>1.6</v>
+        <v>4.7</v>
       </c>
       <c r="AF89" t="n">
-        <v>2.4</v>
+        <v>14.2</v>
       </c>
       <c r="AG89" t="n">
-        <v>0.8</v>
+        <v>10.1</v>
       </c>
       <c r="AH89" t="n">
-        <v>1.3</v>
+        <v>15.9</v>
       </c>
       <c r="AI89" t="n">
-        <v>1.7</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="90">
@@ -12553,19 +12553,19 @@
         <v>13.7</v>
       </c>
       <c r="AB90" t="n">
-        <v>16.8</v>
+        <v>50.4</v>
       </c>
       <c r="AC90" t="n">
-        <v>24.2</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AD90" t="n">
-        <v>18.3</v>
+        <v>54.9</v>
       </c>
       <c r="AE90" t="n">
         <v>0</v>
       </c>
       <c r="AF90" t="n">
-        <v>37.2</v>
+        <v>223.3</v>
       </c>
       <c r="AG90" t="n">
         <v>0</v>
@@ -12574,7 +12574,7 @@
         <v>0</v>
       </c>
       <c r="AI90" t="n">
-        <v>46</v>
+        <v>552</v>
       </c>
     </row>
     <row r="91">
@@ -12690,16 +12690,16 @@
         <v>25.1</v>
       </c>
       <c r="AB91" t="n">
-        <v>36.3</v>
+        <v>108.8</v>
       </c>
       <c r="AC91" t="n">
-        <v>27.9</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="AD91" t="n">
         <v>0</v>
       </c>
       <c r="AE91" t="n">
-        <v>32.1</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AF91" t="n">
         <v>0</v>
@@ -12711,7 +12711,7 @@
         <v>0</v>
       </c>
       <c r="AI91" t="n">
-        <v>23.9</v>
+        <v>287</v>
       </c>
     </row>
     <row r="92">
@@ -12827,25 +12827,25 @@
         <v>0.9</v>
       </c>
       <c r="AB92" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="AC92" t="n">
-        <v>3.2</v>
+        <v>9.5</v>
       </c>
       <c r="AD92" t="n">
-        <v>1.8</v>
+        <v>5.5</v>
       </c>
       <c r="AE92" t="n">
-        <v>0.6</v>
+        <v>1.9</v>
       </c>
       <c r="AF92" t="n">
-        <v>1</v>
+        <v>6.1</v>
       </c>
       <c r="AG92" t="n">
-        <v>0.3</v>
+        <v>3.7</v>
       </c>
       <c r="AH92" t="n">
-        <v>2.2</v>
+        <v>26</v>
       </c>
       <c r="AI92" t="n">
         <v>0</v>
@@ -12967,25 +12967,25 @@
         <v>0</v>
       </c>
       <c r="AC93" t="n">
-        <v>19.7</v>
+        <v>59.1</v>
       </c>
       <c r="AD93" t="n">
         <v>0</v>
       </c>
       <c r="AE93" t="n">
-        <v>16.9</v>
+        <v>50.6</v>
       </c>
       <c r="AF93" t="n">
-        <v>12.3</v>
+        <v>73.8</v>
       </c>
       <c r="AG93" t="n">
-        <v>7.2</v>
+        <v>86</v>
       </c>
       <c r="AH93" t="n">
-        <v>17.6</v>
+        <v>211.5</v>
       </c>
       <c r="AI93" t="n">
-        <v>15.8</v>
+        <v>189.1</v>
       </c>
     </row>
     <row r="94">
@@ -13101,13 +13101,13 @@
         <v>72.7</v>
       </c>
       <c r="AB94" t="n">
-        <v>37.7</v>
+        <v>113</v>
       </c>
       <c r="AC94" t="n">
         <v>0</v>
       </c>
       <c r="AD94" t="n">
-        <v>57.3</v>
+        <v>171.8</v>
       </c>
       <c r="AE94" t="n">
         <v>0</v>
@@ -13116,13 +13116,13 @@
         <v>0</v>
       </c>
       <c r="AG94" t="n">
-        <v>50.8</v>
+        <v>609.1</v>
       </c>
       <c r="AH94" t="n">
         <v>0</v>
       </c>
       <c r="AI94" t="n">
-        <v>38.8</v>
+        <v>465.8</v>
       </c>
     </row>
     <row r="95">
@@ -13238,10 +13238,10 @@
         <v>0</v>
       </c>
       <c r="AB95" t="n">
-        <v>3.2</v>
+        <v>9.6</v>
       </c>
       <c r="AC95" t="n">
-        <v>3.5</v>
+        <v>10.6</v>
       </c>
       <c r="AD95" t="n">
         <v>0</v>
@@ -13250,10 +13250,10 @@
         <v>0</v>
       </c>
       <c r="AF95" t="n">
-        <v>2.1</v>
+        <v>12.6</v>
       </c>
       <c r="AG95" t="n">
-        <v>5.2</v>
+        <v>61.8</v>
       </c>
       <c r="AH95" t="n">
         <v>0</v>
@@ -13375,25 +13375,25 @@
         <v>14.2</v>
       </c>
       <c r="AB96" t="n">
-        <v>40.2</v>
+        <v>120.6</v>
       </c>
       <c r="AC96" t="n">
         <v>0</v>
       </c>
       <c r="AD96" t="n">
-        <v>30.1</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="AE96" t="n">
-        <v>24.2</v>
+        <v>72.5</v>
       </c>
       <c r="AF96" t="n">
         <v>0</v>
       </c>
       <c r="AG96" t="n">
-        <v>17.8</v>
+        <v>213.2</v>
       </c>
       <c r="AH96" t="n">
-        <v>36.4</v>
+        <v>437.2</v>
       </c>
       <c r="AI96" t="n">
         <v>0</v>
@@ -13515,16 +13515,16 @@
         <v>0</v>
       </c>
       <c r="AC97" t="n">
-        <v>36.8</v>
+        <v>110.5</v>
       </c>
       <c r="AD97" t="n">
-        <v>35.3</v>
+        <v>105.9</v>
       </c>
       <c r="AE97" t="n">
-        <v>28.7</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AF97" t="n">
-        <v>1.9</v>
+        <v>11.2</v>
       </c>
       <c r="AG97" t="n">
         <v>0</v>
@@ -13533,7 +13533,7 @@
         <v>0</v>
       </c>
       <c r="AI97" t="n">
-        <v>32.9</v>
+        <v>394.3</v>
       </c>
     </row>
     <row r="98">
@@ -13649,7 +13649,7 @@
         <v>13.9</v>
       </c>
       <c r="AB98" t="n">
-        <v>17.8</v>
+        <v>53.3</v>
       </c>
       <c r="AC98" t="n">
         <v>0</v>
@@ -13658,16 +13658,16 @@
         <v>0</v>
       </c>
       <c r="AE98" t="n">
-        <v>9.6</v>
+        <v>28.7</v>
       </c>
       <c r="AF98" t="n">
-        <v>7.5</v>
+        <v>45.2</v>
       </c>
       <c r="AG98" t="n">
         <v>0</v>
       </c>
       <c r="AH98" t="n">
-        <v>22.2</v>
+        <v>266.5</v>
       </c>
       <c r="AI98" t="n">
         <v>0</v>

</xml_diff>